<commit_message>
Stage 8 fixes: C-021
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Bioanalysis/MV-2023-288/MV-2023-288/MV-2023-288_AssayWorksheet_112723_v03.xlsx
+++ b/output/archive/MerrivossData/Bioanalysis/MV-2023-288/MV-2023-288/MV-2023-288_AssayWorksheet_112723_v03.xlsx
@@ -137,36 +137,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Carole Mills</author>
-  </authors>
-  <commentList>
-    <comment ref="E4" authorId="0" shapeId="0">
-      <text>
-        <t>IV early point is 5 min. Confirm the label on the sampling sheet matches before the bridge is written up.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Helen Marchwood</author>
-  </authors>
-  <commentList>
-    <comment ref="C5" authorId="0" shapeId="0">
-      <text>
-        <t>Re-prepared level kept in the run, original preparation noted on the bench sheet</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -468,7 +438,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MV-2023-288 assay worksheet</t>
+          <t>Merrivoss Bioanalysis Inc, a Tarnovell company: MV-2023-288 assay worksheet</t>
         </is>
       </c>
     </row>
@@ -608,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -621,123 +591,43 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Accession-lot mapping</t>
+          <t>Accession-lot source mapping</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Accession lot</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Dosing lot</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Role in the bridge</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Received</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Storage</t>
+          <t>Source record</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>M23/BIO/06630-01</t>
+          <t>Reference and bridging dosing lots</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Lot A (reference)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Comparator arm</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>10/12/2023</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>-20 °C</t>
+          <t>Signed lot-receipt/analyte cards and dosing-plan allocation under M23/BIO/06630; local lot identifiers remain in those records.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>M23/BIO/06630-02</t>
+          <t>Rat bioanalytical samples</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Lot B (new)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Bridging arm</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>10/12/2023</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>-20 °C</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>M23/BIO/06630-03</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Blank plasma, rat</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Matrix blank and calibration</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>10/09/2023</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>-80 °C</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Dosing formulations are logged against the lot numbers on the dosing record.</t>
+          <t>Sample accession cards identify matrix, anticoagulant, storage and lot/group mapping; these details are not independently reconstructed here.</t>
         </is>
       </c>
     </row>
@@ -753,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -766,157 +656,61 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dosing and sampling protocol</t>
+          <t>Dosing-plan source index</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Dosing lot</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Animals</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Sampling time points (h)</t>
+          <t>Authoritative source / scope</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Administered dose and vehicle</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Lot A (reference)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Oral</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>4 per group</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>0.25, 0.5, 1, 2, 4, 8, 24</t>
+          <t>MV-2023-288 signed dosing plan under M23/BIO/06630: lot/route-specific dose, dose volume, formulation concentration and vehicle composition. Values not transcribed here.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Animal and sampling linkage</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Lot B (new)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Oral</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>4 per group</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>0.25, 0.5, 1, 2, 4, 8, 24</t>
+          <t>Executed dosing/sampling sheets under the same accession: animal identifiers, dose time, nominal/actual collection times and rat matrix.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Exposure-bridge interpretation</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Lot A (reference)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>IV</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>4 per group</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>0.083, 0.25, 0.5, 1, 2, 4, 8, 24</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Lot B (new)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>IV</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>4 per group</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>0.083, 0.25, 0.5, 1, 2, 4, 8, 24</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Sampling was timed from the dose, and the dose-day schedule was agreed with Megan Larkin before the first animal was dosed.</t>
+          <t>MerrivossData/Client_Work/MV-2023-288/MV-2023-288/MV-2023-288_Readout_112723_R1.pptx: comparable exposure retained original efficacy interpretation. This qualitative conclusion is not a numerical equivalence claim.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -926,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -940,173 +734,97 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Matrix acceptance by run</t>
+          <t>Assay-method and run-disposition source index</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Record to consult</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Calibrators</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>QC levels</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Checked by</t>
+          <t>Scope</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>Matrix definition</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>10/25/2023</t>
+          <t>MV-2023-288 signed assay method and sample accession cards under M23/BIO/06630</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Benjamin Ahuja</t>
+          <t>Rat matrix type and anticoagulant must match the method; not transcribed here.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>Calibration range / LLOQ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>10/31/2023</t>
+          <t>Analyte-specific method and calibration records under M23/BIO/06630</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Benjamin Ahuja</t>
+          <t>Range, units, LLOQ and dilution provisions belong to the method, not this index.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>Run criteria</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>11/03/2023</t>
+          <t>Method acceptance section and signed run acceptance sheets</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Met, one level re-prepared</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Helen Marchwood</t>
+          <t>Blank analyte/internal-standard interference, back-calculated calibrator bias/proportion and QC bias/proportions overall/per level.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>Run disposition</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>11/06/2023</t>
+          <t>Original run sheets and any rejected/repeated-run disposition records</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Helen Marchwood</t>
+          <t>Identifiers, exclusions, repeat reasons and sample reanalysis linkage; no Met or accepted status inferred here.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>